<commit_message>
updated file structures and refreshed MIDI circuits
</commit_message>
<xml_diff>
--- a/JustinHours.xlsx
+++ b/JustinHours.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\source\BassMidi\Midi-Bass-Guitar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\Midi-Bass-Guitar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F8CA2D5-0928-46AD-97D0-541B20AF98C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7433F0F4-74C0-449B-8FD4-37C688473889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="W1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="W3" sheetId="3" r:id="rId3"/>
     <sheet name="W4" sheetId="4" r:id="rId4"/>
     <sheet name="W5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sem6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -106,16 +107,47 @@
   </si>
   <si>
     <t xml:space="preserve">Writing Presentation </t>
+  </si>
+  <si>
+    <t>Week#</t>
+  </si>
+  <si>
+    <t>In</t>
+  </si>
+  <si>
+    <t>Out</t>
+  </si>
+  <si>
+    <t>IR Tx Board Design</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Part</t>
+  </si>
+  <si>
+    <t>2Ω Power Resistor</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Bourns/PWR220T-20-2R00F?qs=sGAEpiMZZMtlubZbdhIBIIFas8kKGM5fidmq4iLVFG8%3D</t>
+  </si>
+  <si>
+    <t>IR Rx Board Design</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="##0.000E+0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,16 +155,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -164,11 +210,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -206,11 +290,46 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -496,16 +615,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -520,12 +639,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -541,12 +660,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>0.99999999999999911</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -562,12 +681,12 @@
         <f t="shared" ref="E5:E16" si="0">ABS((D5-C5)*24)</f>
         <v>1.2499999999999982</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -583,12 +702,12 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -604,12 +723,12 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -625,12 +744,12 @@
         <f t="shared" si="0"/>
         <v>1.7499999999999991</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -646,12 +765,12 @@
         <f t="shared" si="0"/>
         <v>0.99999999999999911</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -667,12 +786,12 @@
         <f t="shared" si="0"/>
         <v>1.2499999999999982</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -688,12 +807,12 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -709,12 +828,12 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -730,12 +849,12 @@
         <f t="shared" si="0"/>
         <v>1.7499999999999991</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
@@ -751,12 +870,12 @@
         <f t="shared" si="0"/>
         <v>0.99999999999999911</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
@@ -772,12 +891,12 @@
         <f t="shared" si="0"/>
         <v>1.2499999999999982</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
@@ -793,12 +912,12 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="F16" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C17" s="9"/>
@@ -888,16 +1007,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -912,12 +1031,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -933,12 +1052,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -954,12 +1073,12 @@
         <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
         <v>1.8333333333333321</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -975,12 +1094,12 @@
         <f t="shared" si="0"/>
         <v>2.7499999999999996</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -996,12 +1115,12 @@
         <f t="shared" si="0"/>
         <v>1.416666666666667</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1017,12 +1136,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1038,12 +1157,12 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1059,12 +1178,12 @@
         <f t="shared" si="0"/>
         <v>2.4166666666666661</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1080,12 +1199,12 @@
         <f t="shared" si="0"/>
         <v>2.5000000000000018</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -1101,12 +1220,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1122,12 +1241,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1189,16 +1308,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1213,12 +1332,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1234,12 +1353,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1255,12 +1374,12 @@
         <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
         <v>1.8333333333333321</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1276,12 +1395,12 @@
         <f t="shared" si="0"/>
         <v>2.7499999999999996</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1297,12 +1416,12 @@
         <f t="shared" si="0"/>
         <v>1.416666666666667</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1318,12 +1437,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1339,12 +1458,12 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1360,12 +1479,12 @@
         <f t="shared" si="0"/>
         <v>2.4166666666666661</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1381,12 +1500,12 @@
         <f t="shared" si="0"/>
         <v>2.5000000000000018</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -1402,12 +1521,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1423,12 +1542,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1470,16 +1589,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1494,12 +1613,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1515,12 +1634,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.166666666666667</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1536,12 +1655,12 @@
         <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
         <v>1.6666666666666687</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1557,12 +1676,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1578,12 +1697,12 @@
         <f t="shared" si="0"/>
         <v>1.9166666666666679</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1599,12 +1718,12 @@
         <f t="shared" si="0"/>
         <v>2.4166666666666661</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1620,12 +1739,12 @@
         <f t="shared" si="0"/>
         <v>3.4999999999999982</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1641,12 +1760,12 @@
         <f t="shared" si="0"/>
         <v>2.0833333333333326</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1662,12 +1781,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -1683,12 +1802,12 @@
         <f t="shared" si="0"/>
         <v>2.5000000000000004</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1704,12 +1823,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1751,16 +1870,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1775,12 +1894,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1796,12 +1915,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.166666666666667</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1814,15 +1933,15 @@
         <v>0.61111111111111116</v>
       </c>
       <c r="E5" s="8">
-        <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
+        <f>ABS((D5-C5)*24)</f>
         <v>1.6666666666666687</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1835,15 +1954,15 @@
         <v>0.4861111111111111</v>
       </c>
       <c r="E6" s="8">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E6:E11" si="0">ABS((D6-C6)*24)</f>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1855,10 +1974,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1870,10 +1989,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1885,10 +2004,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1900,10 +2019,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1915,30 +2034,30 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1957,11 +2076,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F12:I12"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="F3:I3"/>
@@ -1969,7 +2083,779 @@
     <mergeCell ref="F5:I5"/>
     <mergeCell ref="F6:I6"/>
     <mergeCell ref="F7:I7"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F12:I12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42FD6328-9B9A-4BF0-A590-87E294C13DA0}">
+  <dimension ref="B3:X29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" style="1"/>
+    <col min="3" max="4" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="17" width="9.140625" style="1"/>
+    <col min="18" max="20" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" style="1"/>
+    <col min="22" max="22" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3">
+        <v>45950</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F4" s="2">
+        <f>ABS((E4-D4)*24)</f>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
+        <v>45950</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F5" s="8">
+        <f>ABS((E5-D5)*24)</f>
+        <v>2.333333333333333</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="S5" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="V5" s="15"/>
+    </row>
+    <row r="6" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="2">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3">
+        <v>45951</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0.48125000000000001</v>
+      </c>
+      <c r="F6" s="8">
+        <f t="shared" ref="F6:F29" si="0">ABS((E6-D6)*24)</f>
+        <v>0.55000000000000071</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="S6" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="T6" s="15"/>
+      <c r="U6" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="V6" s="20"/>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3">
+        <v>45951</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.6875</v>
+      </c>
+      <c r="F7" s="8">
+        <f t="shared" si="0"/>
+        <v>3.5000000000000009</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="15"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+    </row>
+    <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" s="3">
+        <v>45952</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F8" s="8">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
+      <c r="V8"/>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3">
+        <v>45952</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="F9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.8333333333333348</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="S9"/>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3">
+        <v>45953</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="F10" s="8">
+        <f t="shared" si="0"/>
+        <v>2.0000000000000009</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="S10"/>
+      <c r="T10"/>
+      <c r="U10"/>
+      <c r="V10"/>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+      <c r="C11" s="3">
+        <v>45954</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="8">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999996</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
+      <c r="S11"/>
+      <c r="T11"/>
+      <c r="U11"/>
+      <c r="V11"/>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B12" s="21">
+        <v>2</v>
+      </c>
+      <c r="C12" s="22">
+        <v>45957</v>
+      </c>
+      <c r="D12" s="23">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E12" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="24">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25"/>
+      <c r="R12" s="13"/>
+      <c r="S12" s="14"/>
+      <c r="T12" s="14"/>
+      <c r="U12"/>
+      <c r="V12" s="14"/>
+      <c r="W12" s="13"/>
+      <c r="X12" s="13"/>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B13" s="21">
+        <v>2</v>
+      </c>
+      <c r="C13" s="22">
+        <v>45957</v>
+      </c>
+      <c r="D13" s="23">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E13" s="23">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F13" s="24">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25"/>
+      <c r="S13"/>
+      <c r="T13"/>
+      <c r="U13"/>
+      <c r="V13" s="14"/>
+    </row>
+    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B14" s="21">
+        <v>2</v>
+      </c>
+      <c r="C14" s="22">
+        <v>45958</v>
+      </c>
+      <c r="D14" s="23">
+        <v>0.4375</v>
+      </c>
+      <c r="E14" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="24">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="G14" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25"/>
+      <c r="S14"/>
+      <c r="T14"/>
+      <c r="U14"/>
+      <c r="V14"/>
+    </row>
+    <row r="15" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B15" s="21">
+        <v>2</v>
+      </c>
+      <c r="C15" s="22">
+        <v>45958</v>
+      </c>
+      <c r="D15" s="23">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E15" s="23">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F15" s="24">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999982</v>
+      </c>
+      <c r="G15" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+      <c r="S15"/>
+      <c r="T15"/>
+      <c r="U15"/>
+      <c r="V15"/>
+    </row>
+    <row r="16" spans="2:24" x14ac:dyDescent="0.25">
+      <c r="B16" s="21">
+        <v>2</v>
+      </c>
+      <c r="C16" s="22">
+        <v>45959</v>
+      </c>
+      <c r="D16" s="23">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E16" s="23">
+        <v>0.625</v>
+      </c>
+      <c r="F16" s="24">
+        <f t="shared" si="0"/>
+        <v>2.0000000000000009</v>
+      </c>
+      <c r="G16" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
+      <c r="S16"/>
+      <c r="T16"/>
+      <c r="U16"/>
+      <c r="V16"/>
+    </row>
+    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B17" s="21">
+        <v>2</v>
+      </c>
+      <c r="C17" s="22">
+        <v>45959</v>
+      </c>
+      <c r="D17" s="23">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E17" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="F17" s="24">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999996</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
+    </row>
+    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B18" s="21">
+        <v>2</v>
+      </c>
+      <c r="C18" s="22">
+        <v>45960</v>
+      </c>
+      <c r="D18" s="23">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E18" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="F18" s="24">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
+    </row>
+    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B19" s="21">
+        <v>2</v>
+      </c>
+      <c r="C19" s="22">
+        <v>45960</v>
+      </c>
+      <c r="D19" s="23">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E19" s="23">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F19" s="24">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
+      <c r="S19"/>
+      <c r="T19"/>
+      <c r="U19"/>
+      <c r="V19"/>
+    </row>
+    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B20" s="21">
+        <v>2</v>
+      </c>
+      <c r="C20" s="22">
+        <v>45961</v>
+      </c>
+      <c r="D20" s="23">
+        <v>0.4375</v>
+      </c>
+      <c r="E20" s="23">
+        <v>0.5</v>
+      </c>
+      <c r="F20" s="24">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
+      <c r="S20"/>
+      <c r="T20"/>
+      <c r="U20"/>
+      <c r="V20"/>
+    </row>
+    <row r="21" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B21" s="21">
+        <v>2</v>
+      </c>
+      <c r="C21" s="22">
+        <v>45961</v>
+      </c>
+      <c r="D21" s="23">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E21" s="23">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F21" s="24">
+        <f t="shared" si="0"/>
+        <v>1.9999999999999982</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
+    </row>
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B22" s="2">
+        <v>3</v>
+      </c>
+      <c r="C22" s="3">
+        <v>45964</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="8">
+        <f t="shared" si="0"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+    </row>
+    <row r="23" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B23" s="2">
+        <v>3</v>
+      </c>
+      <c r="C23" s="3">
+        <v>45964</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0.53472222222222221</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0.63194444444444442</v>
+      </c>
+      <c r="F23" s="8">
+        <f t="shared" si="0"/>
+        <v>2.333333333333333</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="15"/>
+    </row>
+    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B24" s="2">
+        <v>3</v>
+      </c>
+      <c r="C24" s="3">
+        <v>45965</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0.50347222222222221</v>
+      </c>
+      <c r="F24" s="8">
+        <f t="shared" si="0"/>
+        <v>1.0833333333333335</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+    </row>
+    <row r="25" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B25" s="2">
+        <v>3</v>
+      </c>
+      <c r="C25" s="3">
+        <v>45965</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0.60763888888888884</v>
+      </c>
+      <c r="F25" s="8">
+        <f t="shared" si="0"/>
+        <v>1.583333333333333</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+    </row>
+    <row r="26" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="18"/>
+    </row>
+    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B27" s="2"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G27" s="16"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="18"/>
+    </row>
+    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B28" s="2"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G28" s="16"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="18"/>
+    </row>
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B29" s="2"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="G20:K20"/>
+    <mergeCell ref="G9:K9"/>
+    <mergeCell ref="G10:K10"/>
+    <mergeCell ref="G11:K11"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="G14:K14"/>
+    <mergeCell ref="G15:K15"/>
+    <mergeCell ref="G16:K16"/>
+    <mergeCell ref="G17:K17"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="G19:K19"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
started modeling new fret system
</commit_message>
<xml_diff>
--- a/JustinHours.xlsx
+++ b/JustinHours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\Midi-Bass-Guitar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7433F0F4-74C0-449B-8FD4-37C688473889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8324FA15-8488-426C-8777-BDCF56B60778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -136,7 +136,10 @@
     <t>https://www.mouser.com/ProductDetail/Bourns/PWR220T-20-2R00F?qs=sGAEpiMZZMtlubZbdhIBIIFas8kKGM5fidmq4iLVFG8%3D</t>
   </si>
   <si>
-    <t>IR Rx Board Design</t>
+    <t>IR Rx Circuit Design</t>
+  </si>
+  <si>
+    <t>Bass Fret Bar Design</t>
   </si>
 </sst>
 </file>
@@ -252,7 +255,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -294,24 +297,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -324,7 +309,28 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -615,16 +621,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -639,12 +645,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -660,12 +666,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>0.99999999999999911</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -681,12 +687,12 @@
         <f t="shared" ref="E5:E16" si="0">ABS((D5-C5)*24)</f>
         <v>1.2499999999999982</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -702,12 +708,12 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -723,12 +729,12 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -744,12 +750,12 @@
         <f t="shared" si="0"/>
         <v>1.7499999999999991</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -765,12 +771,12 @@
         <f t="shared" si="0"/>
         <v>0.99999999999999911</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -786,12 +792,12 @@
         <f t="shared" si="0"/>
         <v>1.2499999999999982</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -807,12 +813,12 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -828,12 +834,12 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -849,12 +855,12 @@
         <f t="shared" si="0"/>
         <v>1.7499999999999991</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
@@ -870,12 +876,12 @@
         <f t="shared" si="0"/>
         <v>0.99999999999999911</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
@@ -891,12 +897,12 @@
         <f t="shared" si="0"/>
         <v>1.2499999999999982</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
+      <c r="I15" s="19"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="3">
@@ -912,12 +918,12 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F16" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C17" s="9"/>
@@ -981,21 +987,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F12:I12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1007,16 +1013,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1031,12 +1037,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1052,12 +1058,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1073,12 +1079,12 @@
         <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
         <v>1.8333333333333321</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1094,12 +1100,12 @@
         <f t="shared" si="0"/>
         <v>2.7499999999999996</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1115,12 +1121,12 @@
         <f t="shared" si="0"/>
         <v>1.416666666666667</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1136,12 +1142,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1157,12 +1163,12 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1178,12 +1184,12 @@
         <f t="shared" si="0"/>
         <v>2.4166666666666661</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1199,12 +1205,12 @@
         <f t="shared" si="0"/>
         <v>2.5000000000000018</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -1220,12 +1226,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1241,12 +1247,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1285,18 +1291,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F12:I12"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="F4:I4"/>
     <mergeCell ref="F5:I5"/>
     <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F12:I12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1308,16 +1314,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1332,12 +1338,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1353,12 +1359,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1374,12 +1380,12 @@
         <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
         <v>1.8333333333333321</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1395,12 +1401,12 @@
         <f t="shared" si="0"/>
         <v>2.7499999999999996</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1416,12 +1422,12 @@
         <f t="shared" si="0"/>
         <v>1.416666666666667</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1437,12 +1443,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1458,12 +1464,12 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1479,12 +1485,12 @@
         <f t="shared" si="0"/>
         <v>2.4166666666666661</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1500,12 +1506,12 @@
         <f t="shared" si="0"/>
         <v>2.5000000000000018</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -1521,12 +1527,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1542,12 +1548,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1589,16 +1595,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1613,12 +1619,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1634,12 +1640,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.166666666666667</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1655,12 +1661,12 @@
         <f t="shared" ref="E5:E13" si="0">ABS((D5-C5)*24)</f>
         <v>1.6666666666666687</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1676,12 +1682,12 @@
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1697,12 +1703,12 @@
         <f t="shared" si="0"/>
         <v>1.9166666666666679</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1718,12 +1724,12 @@
         <f t="shared" si="0"/>
         <v>2.4166666666666661</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -1739,12 +1745,12 @@
         <f t="shared" si="0"/>
         <v>3.4999999999999982</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -1760,12 +1766,12 @@
         <f t="shared" si="0"/>
         <v>2.0833333333333326</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -1781,12 +1787,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3">
@@ -1802,12 +1808,12 @@
         <f t="shared" si="0"/>
         <v>2.5000000000000004</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3">
@@ -1823,12 +1829,12 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -1870,16 +1876,16 @@
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -1894,12 +1900,12 @@
       <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
@@ -1915,12 +1921,12 @@
         <f>ABS((D4-C4)*24)</f>
         <v>2.166666666666667</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
@@ -1936,12 +1942,12 @@
         <f>ABS((D5-C5)*24)</f>
         <v>1.6666666666666687</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
@@ -1957,12 +1963,12 @@
         <f t="shared" ref="E6:E11" si="0">ABS((D6-C6)*24)</f>
         <v>2.6666666666666665</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
@@ -1974,10 +1980,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="3">
@@ -1989,10 +1995,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="3">
@@ -2004,10 +2010,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="3">
@@ -2019,10 +2025,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="3">
@@ -2034,30 +2040,30 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
@@ -2125,13 +2131,13 @@
       <c r="F3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
@@ -2150,13 +2156,13 @@
         <f>ABS((E4-D4)*24)</f>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
@@ -2175,21 +2181,21 @@
         <f>ABS((E5-D5)*24)</f>
         <v>2.333333333333333</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="S5" s="15" t="s">
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="S5" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15" t="s">
+      <c r="T5" s="19"/>
+      <c r="U5" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="V5" s="15"/>
+      <c r="V5" s="19"/>
     </row>
     <row r="6" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
@@ -2208,21 +2214,21 @@
         <f t="shared" ref="F6:F29" si="0">ABS((E6-D6)*24)</f>
         <v>0.55000000000000071</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="S6" s="15" t="s">
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="S6" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="T6" s="15"/>
-      <c r="U6" s="19" t="s">
+      <c r="T6" s="19"/>
+      <c r="U6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="20"/>
+      <c r="V6" s="21"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -2241,17 +2247,17 @@
         <f t="shared" si="0"/>
         <v>3.5000000000000009</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
-      <c r="S7" s="15"/>
-      <c r="T7" s="15"/>
-      <c r="U7" s="20"/>
-      <c r="V7" s="20"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="21"/>
+      <c r="V7" s="21"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -2270,13 +2276,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
       <c r="S8"/>
       <c r="T8"/>
       <c r="U8"/>
@@ -2299,13 +2305,13 @@
         <f t="shared" si="0"/>
         <v>1.8333333333333348</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
       <c r="S9"/>
       <c r="T9"/>
       <c r="U9"/>
@@ -2328,13 +2334,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
       <c r="S10"/>
       <c r="T10"/>
       <c r="U10"/>
@@ -2357,42 +2363,42 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="G11" s="15" t="s">
+      <c r="G11" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
       <c r="S11"/>
       <c r="T11"/>
       <c r="U11"/>
       <c r="V11"/>
     </row>
     <row r="12" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B12" s="21">
+      <c r="B12" s="15">
         <v>2</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="16">
         <v>45957</v>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="17">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="17">
         <v>0.5</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="18">
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
       <c r="R12" s="13"/>
       <c r="S12" s="14"/>
       <c r="T12" s="14"/>
@@ -2402,261 +2408,261 @@
       <c r="X12" s="13"/>
     </row>
     <row r="13" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B13" s="21">
+      <c r="B13" s="15">
         <v>2</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="16">
         <v>45957</v>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13" s="17">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="18">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
       <c r="S13"/>
       <c r="T13"/>
       <c r="U13"/>
       <c r="V13" s="14"/>
     </row>
     <row r="14" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B14" s="21">
+      <c r="B14" s="15">
         <v>2</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="16">
         <v>45958</v>
       </c>
-      <c r="D14" s="23">
+      <c r="D14" s="17">
         <v>0.4375</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="17">
         <v>0.5</v>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="18">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="22"/>
+      <c r="J14" s="22"/>
+      <c r="K14" s="22"/>
       <c r="S14"/>
       <c r="T14"/>
       <c r="U14"/>
       <c r="V14"/>
     </row>
     <row r="15" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B15" s="21">
+      <c r="B15" s="15">
         <v>2</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="16">
         <v>45958</v>
       </c>
-      <c r="D15" s="23">
+      <c r="D15" s="17">
         <v>0.52083333333333337</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15" s="17">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="18">
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="G15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
       <c r="S15"/>
       <c r="T15"/>
       <c r="U15"/>
       <c r="V15"/>
     </row>
     <row r="16" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B16" s="21">
+      <c r="B16" s="15">
         <v>2</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="16">
         <v>45959</v>
       </c>
-      <c r="D16" s="23">
+      <c r="D16" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E16" s="17">
         <v>0.625</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="18">
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="G16" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
       <c r="S16"/>
       <c r="T16"/>
       <c r="U16"/>
       <c r="V16"/>
     </row>
     <row r="17" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B17" s="21">
+      <c r="B17" s="15">
         <v>2</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="16">
         <v>45959</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="17">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="17">
         <v>0.5</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="18">
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="G17" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
       <c r="V17"/>
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B18" s="21">
+      <c r="B18" s="15">
         <v>2</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="16">
         <v>45960</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="17">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E18" s="23">
+      <c r="E18" s="17">
         <v>0.5</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="18">
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G18" s="25" t="s">
+      <c r="G18" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
       <c r="S18"/>
       <c r="T18"/>
       <c r="U18"/>
       <c r="V18"/>
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B19" s="21">
+      <c r="B19" s="15">
         <v>2</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="16">
         <v>45960</v>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="17">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="18">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
       <c r="S19"/>
       <c r="T19"/>
       <c r="U19"/>
       <c r="V19"/>
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B20" s="21">
+      <c r="B20" s="15">
         <v>2</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="16">
         <v>45961</v>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="17">
         <v>0.4375</v>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="17">
         <v>0.5</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="18">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
       <c r="S20"/>
       <c r="T20"/>
       <c r="U20"/>
       <c r="V20"/>
     </row>
     <row r="21" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B21" s="21">
+      <c r="B21" s="15">
         <v>2</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="16">
         <v>45961</v>
       </c>
-      <c r="D21" s="23">
+      <c r="D21" s="17">
         <v>0.52083333333333337</v>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="17">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="18">
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G21" s="25" t="s">
+      <c r="G21" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
@@ -2675,13 +2681,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="G22" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B23" s="2">
@@ -2700,13 +2706,13 @@
         <f t="shared" si="0"/>
         <v>2.333333333333333</v>
       </c>
-      <c r="G23" s="15" t="s">
+      <c r="G23" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B24" s="2">
@@ -2725,13 +2731,13 @@
         <f t="shared" si="0"/>
         <v>1.0833333333333335</v>
       </c>
-      <c r="G24" s="15" t="s">
+      <c r="G24" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
     </row>
     <row r="25" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B25" s="2">
@@ -2750,58 +2756,80 @@
         <f t="shared" si="0"/>
         <v>1.583333333333333</v>
       </c>
-      <c r="G25" s="15" t="s">
+      <c r="G25" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
     </row>
     <row r="26" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B26" s="2"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
+      <c r="B26" s="2">
+        <v>3</v>
+      </c>
+      <c r="C26" s="3">
+        <v>45966</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0.40277777777777779</v>
+      </c>
       <c r="F26" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G26" s="16"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="18"/>
+        <v>0.66666666666666696</v>
+      </c>
+      <c r="G26" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B27" s="2"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="2"/>
+      <c r="B27" s="2">
+        <v>3</v>
+      </c>
+      <c r="C27" s="3">
+        <v>45966</v>
+      </c>
+      <c r="D27" s="4">
+        <v>0.40277777777777779</v>
+      </c>
       <c r="E27" s="2"/>
       <c r="F27" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G27" s="16"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="18"/>
+        <v>9.6666666666666679</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="25"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B28" s="2"/>
-      <c r="C28" s="3"/>
+      <c r="B28" s="2">
+        <v>3</v>
+      </c>
+      <c r="C28" s="3">
+        <v>45966</v>
+      </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="18"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="25"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="2"/>
@@ -2812,24 +2840,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G29" s="16"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="18"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
     <mergeCell ref="G20:K20"/>
     <mergeCell ref="G9:K9"/>
     <mergeCell ref="G10:K10"/>
@@ -2842,15 +2869,16 @@
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="G18:K18"/>
     <mergeCell ref="G19:K19"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>

<commit_message>
some cad work and updated midi note charts
</commit_message>
<xml_diff>
--- a/JustinHours.xlsx
+++ b/JustinHours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\Midi-Bass-Guitar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8324FA15-8488-426C-8777-BDCF56B60778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51733FA4-9789-4260-85EF-C04FE5BB0722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="35">
   <si>
     <t>Date</t>
   </si>
@@ -140,6 +140,12 @@
   </si>
   <si>
     <t>Bass Fret Bar Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment Maintenance </t>
+  </si>
+  <si>
+    <t>Administration</t>
   </si>
 </sst>
 </file>
@@ -255,7 +261,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -312,15 +318,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -330,8 +327,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -987,21 +990,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="F14:I14"/>
     <mergeCell ref="F15:I15"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="F11:I11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1291,18 +1294,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="F11:I11"/>
     <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2101,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42FD6328-9B9A-4BF0-A590-87E294C13DA0}">
-  <dimension ref="B3:X29"/>
+  <dimension ref="B3:X45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
@@ -2225,10 +2228,10 @@
         <v>29</v>
       </c>
       <c r="T6" s="19"/>
-      <c r="U6" s="20" t="s">
+      <c r="U6" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="21"/>
+      <c r="V6" s="25"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -2256,8 +2259,8 @@
       <c r="K7" s="19"/>
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
-      <c r="U7" s="21"/>
-      <c r="V7" s="21"/>
+      <c r="U7" s="25"/>
+      <c r="V7" s="25"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -2276,13 +2279,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
       <c r="S8"/>
       <c r="T8"/>
       <c r="U8"/>
@@ -2305,13 +2308,13 @@
         <f t="shared" si="0"/>
         <v>1.8333333333333348</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
       <c r="S9"/>
       <c r="T9"/>
       <c r="U9"/>
@@ -2392,13 +2395,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
       <c r="R12" s="13"/>
       <c r="S12" s="14"/>
       <c r="T12" s="14"/>
@@ -2424,13 +2427,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="22"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
       <c r="S13"/>
       <c r="T13"/>
       <c r="U13"/>
@@ -2453,13 +2456,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
       <c r="S14"/>
       <c r="T14"/>
       <c r="U14"/>
@@ -2482,13 +2485,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G15" s="22" t="s">
+      <c r="G15" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
       <c r="S15"/>
       <c r="T15"/>
       <c r="U15"/>
@@ -2511,13 +2514,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
       <c r="S16"/>
       <c r="T16"/>
       <c r="U16"/>
@@ -2540,13 +2543,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
@@ -2569,13 +2572,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
       <c r="S18"/>
       <c r="T18"/>
       <c r="U18"/>
@@ -2598,13 +2601,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
       <c r="S19"/>
       <c r="T19"/>
       <c r="U19"/>
@@ -2627,13 +2630,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G20" s="22" t="s">
+      <c r="G20" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
       <c r="S20"/>
       <c r="T20"/>
       <c r="U20"/>
@@ -2656,13 +2659,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
@@ -2781,13 +2784,13 @@
         <f t="shared" si="0"/>
         <v>0.66666666666666696</v>
       </c>
-      <c r="G26" s="26" t="s">
+      <c r="G26" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B27" s="2">
@@ -2799,18 +2802,20 @@
       <c r="D27" s="4">
         <v>0.40277777777777779</v>
       </c>
-      <c r="E27" s="2"/>
+      <c r="E27" s="4">
+        <v>0.5</v>
+      </c>
       <c r="F27" s="8">
         <f t="shared" si="0"/>
-        <v>9.6666666666666679</v>
-      </c>
-      <c r="G27" s="23" t="s">
+        <v>2.333333333333333</v>
+      </c>
+      <c r="G27" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
-      <c r="J27" s="24"/>
-      <c r="K27" s="25"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="22"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
@@ -2819,44 +2824,357 @@
       <c r="C28" s="3">
         <v>45966</v>
       </c>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+      <c r="D28" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E28" s="4">
+        <v>0.66666666666666663</v>
+      </c>
       <c r="F28" s="8">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="G28" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="22"/>
+    </row>
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B29" s="2">
+        <v>3</v>
+      </c>
+      <c r="C29" s="3">
+        <v>45967</v>
+      </c>
+      <c r="D29" s="4">
+        <v>0.5625</v>
+      </c>
+      <c r="E29" s="4">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="F29" s="8">
+        <f t="shared" si="0"/>
+        <v>2.0000000000000009</v>
+      </c>
+      <c r="G29" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H29" s="21"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="22"/>
+    </row>
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B30" s="2">
+        <v>3</v>
+      </c>
+      <c r="C30" s="3">
+        <v>45968</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="E30" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F30" s="8">
+        <f t="shared" ref="F30:F45" si="1">ABS((E30-D30)*24)</f>
+        <v>3</v>
+      </c>
+      <c r="G30" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="22"/>
+    </row>
+    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B31" s="2">
+        <v>3</v>
+      </c>
+      <c r="C31" s="3">
+        <v>45968</v>
+      </c>
+      <c r="D31" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E31" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="F31" s="8">
+        <f t="shared" si="1"/>
+        <v>2.0000000000000009</v>
+      </c>
+      <c r="G31" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H31" s="21"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="22"/>
+    </row>
+    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B32" s="2">
+        <v>4</v>
+      </c>
+      <c r="C32" s="3">
+        <v>45971</v>
+      </c>
+      <c r="D32" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E32" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="F32" s="8">
+        <f t="shared" si="1"/>
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="G32" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="22"/>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B33" s="2">
+        <v>4</v>
+      </c>
+      <c r="C33" s="3">
+        <v>45971</v>
+      </c>
+      <c r="D33" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E33" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="F33" s="8">
+        <f t="shared" si="1"/>
+        <v>2.0000000000000009</v>
+      </c>
+      <c r="G33" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="22"/>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B34" s="2"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="8">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G28" s="23"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="25"/>
-    </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B29" s="2"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="8">
-        <f t="shared" si="0"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="21"/>
+      <c r="K34" s="22"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B35" s="2"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="8">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G29" s="23"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="25"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="22"/>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B36" s="2"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G36" s="20"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="21"/>
+      <c r="K36" s="22"/>
+    </row>
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B37" s="2"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G37" s="20"/>
+      <c r="H37" s="21"/>
+      <c r="I37" s="21"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="22"/>
+    </row>
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B38" s="2"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="20"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="22"/>
+    </row>
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B39" s="2"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G39" s="20"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="22"/>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B40" s="2"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G40" s="20"/>
+      <c r="H40" s="21"/>
+      <c r="I40" s="21"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="22"/>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B41" s="2"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G41" s="20"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="21"/>
+      <c r="J41" s="21"/>
+      <c r="K41" s="22"/>
+    </row>
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B42" s="2"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G42" s="20"/>
+      <c r="H42" s="21"/>
+      <c r="I42" s="21"/>
+      <c r="J42" s="21"/>
+      <c r="K42" s="22"/>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B43" s="2"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G43" s="20"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="21"/>
+      <c r="J43" s="21"/>
+      <c r="K43" s="22"/>
+    </row>
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B44" s="2"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G44" s="20"/>
+      <c r="H44" s="21"/>
+      <c r="I44" s="21"/>
+      <c r="J44" s="21"/>
+      <c r="K44" s="22"/>
+    </row>
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B45" s="2"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G45" s="20"/>
+      <c r="H45" s="21"/>
+      <c r="I45" s="21"/>
+      <c r="J45" s="21"/>
+      <c r="K45" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
+  <mergeCells count="47">
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
     <mergeCell ref="G20:K20"/>
     <mergeCell ref="G9:K9"/>
     <mergeCell ref="G10:K10"/>
@@ -2869,16 +3187,15 @@
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="G18:K18"/>
     <mergeCell ref="G19:K19"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>

<commit_message>
updated Universal Master schematic
</commit_message>
<xml_diff>
--- a/JustinHours.xlsx
+++ b/JustinHours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\Midi-Bass-Guitar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C9A2A1-4427-46D2-8C8B-6C2C8ACB558A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B9ED207-F3A5-4B2C-B78C-E5697CAC5DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="38">
   <si>
     <t>Date</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Designing SUDO code</t>
+  </si>
+  <si>
+    <t>Universal Master circuit design</t>
   </si>
 </sst>
 </file>
@@ -333,14 +336,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -996,21 +999,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="F14:I14"/>
     <mergeCell ref="F15:I15"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="F11:I11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1300,18 +1303,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="F11:I11"/>
     <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2234,10 +2237,10 @@
         <v>29</v>
       </c>
       <c r="T6" s="19"/>
-      <c r="U6" s="23" t="s">
+      <c r="U6" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="24"/>
+      <c r="V6" s="25"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -2265,8 +2268,8 @@
       <c r="K7" s="19"/>
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
-      <c r="U7" s="24"/>
-      <c r="V7" s="24"/>
+      <c r="U7" s="25"/>
+      <c r="V7" s="25"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -2401,13 +2404,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
       <c r="R12" s="13"/>
       <c r="S12" s="14"/>
       <c r="T12" s="14"/>
@@ -2433,13 +2436,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
       <c r="S13"/>
       <c r="T13"/>
       <c r="U13"/>
@@ -2462,13 +2465,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
       <c r="S14"/>
       <c r="T14"/>
       <c r="U14"/>
@@ -2491,13 +2494,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="G15" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
       <c r="S15"/>
       <c r="T15"/>
       <c r="U15"/>
@@ -2520,13 +2523,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="G16" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
       <c r="S16"/>
       <c r="T16"/>
       <c r="U16"/>
@@ -2549,13 +2552,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="G17" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
@@ -2578,13 +2581,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G18" s="25" t="s">
+      <c r="G18" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
       <c r="S18"/>
       <c r="T18"/>
       <c r="U18"/>
@@ -2607,13 +2610,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
       <c r="S19"/>
       <c r="T19"/>
       <c r="U19"/>
@@ -2636,13 +2639,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
       <c r="S20"/>
       <c r="T20"/>
       <c r="U20"/>
@@ -2665,13 +2668,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G21" s="25" t="s">
+      <c r="G21" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
@@ -3024,30 +3027,50 @@
       <c r="K35" s="22"/>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B36" s="2"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="B36" s="2">
+        <v>4</v>
+      </c>
+      <c r="C36" s="3">
+        <v>45973</v>
+      </c>
+      <c r="D36" s="4">
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="E36" s="4">
+        <v>0.51041666666666663</v>
+      </c>
       <c r="F36" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G36" s="20"/>
+        <v>1.1499999999999986</v>
+      </c>
+      <c r="G36" s="20" t="s">
+        <v>35</v>
+      </c>
       <c r="H36" s="21"/>
       <c r="I36" s="21"/>
       <c r="J36" s="21"/>
       <c r="K36" s="22"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B37" s="2"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
+      <c r="B37" s="2">
+        <v>4</v>
+      </c>
+      <c r="C37" s="3">
+        <v>45973</v>
+      </c>
+      <c r="D37" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E37" s="4">
+        <v>0.61805555555555558</v>
+      </c>
       <c r="F37" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G37" s="20"/>
+        <v>1.8333333333333348</v>
+      </c>
+      <c r="G37" s="20" t="s">
+        <v>37</v>
+      </c>
       <c r="H37" s="21"/>
       <c r="I37" s="21"/>
       <c r="J37" s="21"/>
@@ -3175,15 +3198,32 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
     <mergeCell ref="G20:K20"/>
     <mergeCell ref="G9:K9"/>
     <mergeCell ref="G10:K10"/>
@@ -3196,32 +3236,15 @@
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="G18:K18"/>
     <mergeCell ref="G19:K19"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="G44:K44"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>

<commit_message>
made new master, pluck and fret circuits
</commit_message>
<xml_diff>
--- a/JustinHours.xlsx
+++ b/JustinHours.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juxin\Documents\Midi-Bass-Guitar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B9ED207-F3A5-4B2C-B78C-E5697CAC5DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B973A21-877C-42CC-A569-00FBF2F7A1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -155,6 +155,18 @@
   </si>
   <si>
     <t>Universal Master circuit design</t>
+  </si>
+  <si>
+    <t>8Pin Molex</t>
+  </si>
+  <si>
+    <t>2Pin Molex</t>
+  </si>
+  <si>
+    <t>Fret circuit design</t>
+  </si>
+  <si>
+    <t>Pluck circuit design</t>
   </si>
 </sst>
 </file>
@@ -270,7 +282,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -336,14 +348,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -999,21 +1023,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="F6:I6"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F12:I12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1303,18 +1327,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F12:I12"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="F4:I4"/>
     <mergeCell ref="F5:I5"/>
     <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F12:I12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2237,10 +2261,10 @@
         <v>29</v>
       </c>
       <c r="T6" s="19"/>
-      <c r="U6" s="24" t="s">
+      <c r="U6" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="V6" s="25"/>
+      <c r="V6" s="24"/>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
@@ -2268,8 +2292,8 @@
       <c r="K7" s="19"/>
       <c r="S7" s="19"/>
       <c r="T7" s="19"/>
-      <c r="U7" s="25"/>
-      <c r="V7" s="25"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="24"/>
     </row>
     <row r="8" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
@@ -2295,10 +2319,14 @@
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
       <c r="K8" s="19"/>
-      <c r="S8"/>
-      <c r="T8"/>
-      <c r="U8"/>
-      <c r="V8"/>
+      <c r="S8" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="T8" s="26"/>
+      <c r="U8" s="26">
+        <v>430450810</v>
+      </c>
+      <c r="V8" s="26"/>
     </row>
     <row r="9" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
@@ -2324,10 +2352,14 @@
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
-      <c r="S9"/>
-      <c r="T9"/>
-      <c r="U9"/>
-      <c r="V9"/>
+      <c r="S9" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="T9" s="26"/>
+      <c r="U9" s="26">
+        <v>430450200</v>
+      </c>
+      <c r="V9" s="26"/>
     </row>
     <row r="10" spans="2:24" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
@@ -2404,13 +2436,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G12" s="23" t="s">
+      <c r="G12" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25"/>
       <c r="R12" s="13"/>
       <c r="S12" s="14"/>
       <c r="T12" s="14"/>
@@ -2436,13 +2468,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25"/>
       <c r="S13"/>
       <c r="T13"/>
       <c r="U13"/>
@@ -2465,13 +2497,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25"/>
       <c r="S14"/>
       <c r="T14"/>
       <c r="U14"/>
@@ -2494,13 +2526,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G15" s="23" t="s">
+      <c r="G15" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
       <c r="S15"/>
       <c r="T15"/>
       <c r="U15"/>
@@ -2523,13 +2555,13 @@
         <f t="shared" si="0"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25"/>
       <c r="S16"/>
       <c r="T16"/>
       <c r="U16"/>
@@ -2552,13 +2584,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999996</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
       <c r="S17"/>
       <c r="T17"/>
       <c r="U17"/>
@@ -2581,13 +2613,13 @@
         <f t="shared" si="0"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G18" s="23" t="s">
+      <c r="G18" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
       <c r="S18"/>
       <c r="T18"/>
       <c r="U18"/>
@@ -2610,13 +2642,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G19" s="23" t="s">
+      <c r="G19" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
       <c r="S19"/>
       <c r="T19"/>
       <c r="U19"/>
@@ -2639,13 +2671,13 @@
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="G20" s="23" t="s">
+      <c r="G20" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="25"/>
       <c r="S20"/>
       <c r="T20"/>
       <c r="U20"/>
@@ -2668,13 +2700,13 @@
         <f t="shared" si="0"/>
         <v>1.9999999999999982</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="G21" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="25"/>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
@@ -2927,247 +2959,301 @@
       <c r="K31" s="22"/>
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B32" s="2">
+      <c r="B32" s="15">
         <v>4</v>
       </c>
-      <c r="C32" s="3">
+      <c r="C32" s="16">
         <v>45971</v>
       </c>
-      <c r="D32" s="4">
+      <c r="D32" s="17">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32" s="17">
         <v>0.5</v>
       </c>
-      <c r="F32" s="8">
+      <c r="F32" s="18">
         <f t="shared" si="1"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="G32" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="22"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="29"/>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B33" s="2">
+      <c r="B33" s="15">
         <v>4</v>
       </c>
-      <c r="C33" s="3">
+      <c r="C33" s="16">
         <v>45971</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D33" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="17">
         <v>0.625</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="18">
         <f t="shared" si="1"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="G33" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="22"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="29"/>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B34" s="2">
+      <c r="B34" s="15">
         <v>4</v>
       </c>
-      <c r="C34" s="3">
+      <c r="C34" s="16">
         <v>45972</v>
       </c>
-      <c r="D34" s="4">
+      <c r="D34" s="17">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E34" s="4">
+      <c r="E34" s="17">
         <v>0.5</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="18">
         <f t="shared" si="1"/>
         <v>1.0000000000000004</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="H34" s="21"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21"/>
-      <c r="K34" s="22"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="28"/>
+      <c r="K34" s="29"/>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B35" s="2">
+      <c r="B35" s="15">
         <v>4</v>
       </c>
-      <c r="C35" s="3">
+      <c r="C35" s="16">
         <v>45972</v>
       </c>
-      <c r="D35" s="4">
+      <c r="D35" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E35" s="4">
+      <c r="E35" s="17">
         <v>0.625</v>
       </c>
-      <c r="F35" s="8">
+      <c r="F35" s="18">
         <f t="shared" si="1"/>
         <v>2.0000000000000009</v>
       </c>
-      <c r="G35" s="20" t="s">
+      <c r="G35" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="H35" s="21"/>
-      <c r="I35" s="21"/>
-      <c r="J35" s="21"/>
-      <c r="K35" s="22"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="28"/>
+      <c r="K35" s="29"/>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B36" s="2">
+      <c r="B36" s="15">
         <v>4</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36" s="16">
         <v>45973</v>
       </c>
-      <c r="D36" s="4">
+      <c r="D36" s="17">
         <v>0.46250000000000002</v>
       </c>
-      <c r="E36" s="4">
+      <c r="E36" s="17">
         <v>0.51041666666666663</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="18">
         <f t="shared" si="1"/>
         <v>1.1499999999999986</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="G36" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="H36" s="21"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="21"/>
-      <c r="K36" s="22"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="29"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B37" s="2">
+      <c r="B37" s="15">
         <v>4</v>
       </c>
-      <c r="C37" s="3">
+      <c r="C37" s="16">
         <v>45973</v>
       </c>
-      <c r="D37" s="4">
+      <c r="D37" s="17">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E37" s="17">
         <v>0.61805555555555558</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="18">
         <f t="shared" si="1"/>
         <v>1.8333333333333348</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="G37" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="H37" s="21"/>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="22"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="29"/>
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B38" s="2"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="8">
+      <c r="B38" s="15">
+        <v>4</v>
+      </c>
+      <c r="C38" s="16">
+        <v>45974</v>
+      </c>
+      <c r="D38" s="17">
+        <v>0.4513888888888889</v>
+      </c>
+      <c r="E38" s="17">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="F38" s="18">
+        <f t="shared" si="1"/>
+        <v>0.66666666666666696</v>
+      </c>
+      <c r="G38" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="29"/>
+    </row>
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B39" s="15">
+        <v>4</v>
+      </c>
+      <c r="C39" s="16">
+        <v>45974</v>
+      </c>
+      <c r="D39" s="17">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="E39" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="F39" s="18">
+        <f t="shared" si="1"/>
+        <v>0.49999999999999956</v>
+      </c>
+      <c r="G39" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="H39" s="28"/>
+      <c r="I39" s="28"/>
+      <c r="J39" s="28"/>
+      <c r="K39" s="29"/>
+    </row>
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B40" s="15">
+        <v>4</v>
+      </c>
+      <c r="C40" s="16">
+        <v>45974</v>
+      </c>
+      <c r="D40" s="17">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E40" s="17">
+        <v>0.5625</v>
+      </c>
+      <c r="F40" s="18">
+        <f t="shared" si="1"/>
+        <v>0.50000000000000089</v>
+      </c>
+      <c r="G40" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="29"/>
+    </row>
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B41" s="15">
+        <v>4</v>
+      </c>
+      <c r="C41" s="16">
+        <v>45974</v>
+      </c>
+      <c r="D41" s="17">
+        <v>0.5625</v>
+      </c>
+      <c r="E41" s="17">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="F41" s="18">
+        <f t="shared" si="1"/>
+        <v>0.99999999999999911</v>
+      </c>
+      <c r="G41" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="H41" s="28"/>
+      <c r="I41" s="28"/>
+      <c r="J41" s="28"/>
+      <c r="K41" s="29"/>
+    </row>
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B42" s="15">
+        <v>4</v>
+      </c>
+      <c r="C42" s="16">
+        <v>45974</v>
+      </c>
+      <c r="D42" s="17">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E42" s="17">
+        <v>0.625</v>
+      </c>
+      <c r="F42" s="18">
+        <f t="shared" si="1"/>
+        <v>0.50000000000000089</v>
+      </c>
+      <c r="G42" s="27" t="s">
+        <v>41</v>
+      </c>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="29"/>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B43" s="15">
+        <v>4</v>
+      </c>
+      <c r="C43" s="16"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G38" s="20"/>
-      <c r="H38" s="21"/>
-      <c r="I38" s="21"/>
-      <c r="J38" s="21"/>
-      <c r="K38" s="22"/>
-    </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B39" s="2"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G39" s="20"/>
-      <c r="H39" s="21"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="21"/>
-      <c r="K39" s="22"/>
-    </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B40" s="2"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G40" s="20"/>
-      <c r="H40" s="21"/>
-      <c r="I40" s="21"/>
-      <c r="J40" s="21"/>
-      <c r="K40" s="22"/>
-    </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B41" s="2"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G41" s="20"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="21"/>
-      <c r="J41" s="21"/>
-      <c r="K41" s="22"/>
-    </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B42" s="2"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G42" s="20"/>
-      <c r="H42" s="21"/>
-      <c r="I42" s="21"/>
-      <c r="J42" s="21"/>
-      <c r="K42" s="22"/>
-    </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B43" s="2"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G43" s="20"/>
-      <c r="H43" s="21"/>
-      <c r="I43" s="21"/>
-      <c r="J43" s="21"/>
-      <c r="K43" s="22"/>
+      <c r="G43" s="27"/>
+      <c r="H43" s="28"/>
+      <c r="I43" s="28"/>
+      <c r="J43" s="28"/>
+      <c r="K43" s="29"/>
     </row>
     <row r="44" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B44" s="2"/>
+      <c r="B44" s="2">
+        <v>4</v>
+      </c>
       <c r="C44" s="3"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -3182,7 +3268,9 @@
       <c r="K44" s="22"/>
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B45" s="2"/>
+      <c r="B45" s="2">
+        <v>4</v>
+      </c>
       <c r="C45" s="3"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -3197,33 +3285,19 @@
       <c r="K45" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="47">
-    <mergeCell ref="G45:K45"/>
-    <mergeCell ref="G40:K40"/>
-    <mergeCell ref="G41:K41"/>
-    <mergeCell ref="G42:K42"/>
-    <mergeCell ref="G43:K43"/>
-    <mergeCell ref="G44:K44"/>
-    <mergeCell ref="G35:K35"/>
-    <mergeCell ref="G36:K36"/>
-    <mergeCell ref="G37:K37"/>
-    <mergeCell ref="G38:K38"/>
-    <mergeCell ref="G39:K39"/>
-    <mergeCell ref="G30:K30"/>
-    <mergeCell ref="G31:K31"/>
-    <mergeCell ref="G32:K32"/>
-    <mergeCell ref="G33:K33"/>
-    <mergeCell ref="G34:K34"/>
-    <mergeCell ref="U5:V5"/>
-    <mergeCell ref="U6:V7"/>
-    <mergeCell ref="G8:K8"/>
-    <mergeCell ref="S5:T5"/>
-    <mergeCell ref="S6:T7"/>
-    <mergeCell ref="G3:K3"/>
-    <mergeCell ref="G4:K4"/>
-    <mergeCell ref="G5:K5"/>
-    <mergeCell ref="G6:K6"/>
-    <mergeCell ref="G7:K7"/>
+  <mergeCells count="51">
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
     <mergeCell ref="G20:K20"/>
     <mergeCell ref="G9:K9"/>
     <mergeCell ref="G10:K10"/>
@@ -3236,15 +3310,33 @@
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="G18:K18"/>
     <mergeCell ref="G19:K19"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G28:K28"/>
-    <mergeCell ref="G29:K29"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="G4:K4"/>
+    <mergeCell ref="G5:K5"/>
+    <mergeCell ref="G6:K6"/>
+    <mergeCell ref="G7:K7"/>
+    <mergeCell ref="U5:V5"/>
+    <mergeCell ref="U6:V7"/>
+    <mergeCell ref="G8:K8"/>
+    <mergeCell ref="S5:T5"/>
+    <mergeCell ref="S6:T7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="G30:K30"/>
+    <mergeCell ref="G31:K31"/>
+    <mergeCell ref="G32:K32"/>
+    <mergeCell ref="G33:K33"/>
+    <mergeCell ref="G34:K34"/>
+    <mergeCell ref="G35:K35"/>
+    <mergeCell ref="G36:K36"/>
+    <mergeCell ref="G37:K37"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="G39:K39"/>
+    <mergeCell ref="G45:K45"/>
+    <mergeCell ref="G40:K40"/>
+    <mergeCell ref="G41:K41"/>
+    <mergeCell ref="G42:K42"/>
+    <mergeCell ref="G43:K43"/>
+    <mergeCell ref="G44:K44"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="U6" r:id="rId1" xr:uid="{C20C1F99-1D02-49D1-A4F0-3A6675C39A16}"/>

</xml_diff>